<commit_message>
feat(F-NAR-019): ATOM-DIF.PAR.001-02 Le seau dans le sable chaud
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.PAR.001-02.xlsx
+++ b/stories/arbres/ATOM-DIF.PAR.001-02.xlsx
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Le puits du seau rouge</t>
+          <t>Le seau dans le sable chaud</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>parc, bac à sable, couverture à carreaux</t>
+          <t>parc, bac à sable, couverture à carreaux, banc, oiseau gris, seau rouge, pelle jaune, gourde</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Nino veut un puits dans le sable pour le seau rouge. Mila parle peu. Il lui tend le seau. Ils creusent. L'eau de la gourde tombe dans le puits.</t>
+          <t>Le seau rouge tape le bac. Près du banc, un éclat de banc brille. Un oiseau gris picore. Nino veut un puits, maintenant, pour le seau. Mila parle peu. Il fonce, explique trop, le seau penche. Sourire parti. Il refuse de foncer, tend le seau, attend. Merci vécu. Gourde trop vite. Il s'arrête, lit l'éclat. Un éclat de banc tient près de l'oiseau.</t>
         </is>
       </c>
     </row>
@@ -1189,17 +1189,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une cigale chante tout près du bac. Le sable sent encore le soleil. Un oiseau gris picore près du banc. Papa pose le sac de goûter. Le sac fait un bruit de papier. Maman déplie une couverture à carreaux. Les carreaux sont bleus et blancs. Tu as entendu la cigale, Nino ? Elle chante fort. Le sable est encore chaud. Je veux un puits. Pour le seau rouge. Un puits dans le bac ? Oui. Bien creux. En ce moment, Nino s'assoit près du bac. Le seau rouge est tiède. Une pelle jaune est à côté. Le manche est un peu rêche. Mila est déjà là. Elle parle peu. Elle regarde ses mains. Le sable y brille un peu.</t>
+          <t>Le plastique du seau tape le rebord du bac. Ça fait toc, court et chaud. J'ai entendu le toc. Près du bac, Nino ? Oui, papa. Le sable sent le soleil. Papa pose le sac de goûter. Le sac fait un bruit de papier. Je déplie la couverture à carreaux. Les carreaux sont bleus et blancs. Elle est tiède, maman. Tu la sens, sous les genoux ? Oui, maman. Un oiseau gris picore près du banc. Au bord du bois, un éclat de banc brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une cigale chante près des arbres. Elle chante fort. Le sable est chaud, Nino ? Oui, il brûle un peu. Je veux un puits, maintenant ! Un puits pour le seau rouge. Un puits dans le bac ? Oui. Bien creux. En ce moment, Nino s'assoit près du bac. Le seau rouge est tiède. Une pelle jaune est à côté. Le manche est un peu rêche. Il gratte, papa. Tu tiens la pelle, Nino ? Oui, papa. Mila arrive près du bac. Elle marche sans bruit. Tu creuses avec moi ? Mila ne dit rien. Elle regarde ses mains. Le sable y luit un peu. On fait un puits. Nino ouvre la bouche trop vite. Les mots montent. Tu vois Mila, Nino ? Oui, papa.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une cigale chante tout près du bac. Le sable sent encore le soleil. Un oiseau gris picore près du banc. Papa pose le sac de goûter. Le sac fait un bruit de papier. Maman déplie une couverture à carreaux. Les carreaux sont bleus et blancs. Tu as entendu la cigale, Nino ? Elle chante fort. Le sable est encore chaud. Je veux un puits. Pour le seau rouge. Un puits dans le bac ? Oui. Bien creux. En ce moment, Nino s'assoit près du bac. Le seau rouge est tiède. Une pelle jaune est à côté. Le manche est un peu rêche. Mila est déjà là. Elle parle peu. Elle regarde ses mains. Le sable y brille un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Le plastique du seau tape le rebord du bac. Ça fait toc, court et chaud. J'ai entendu le toc. Près du bac, Nino ? Oui, papa. Le sable sent le soleil. Papa pose le sac de goûter. Le sac fait un bruit de papier. Je déplie la couverture à carreaux. Les carreaux sont bleus et blancs. Elle est tiède, maman. Tu la sens, sous les genoux ? Oui, maman. Un oiseau gris picore près du banc. Au bord du bois, un &lt;emphasis level="moderate"&gt;éclat de banc&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une cigale chante près des arbres. Elle chante fort. Le sable est chaud, Nino ? Oui, il brûle un peu. Je veux un puits, maintenant ! Un puits pour le seau rouge. Un puits dans le bac ? Oui. Bien creux. En ce moment, Nino s'assoit près du bac. Le seau rouge est tiède. Une pelle jaune est à côté. Le manche est un peu rêche. Il gratte, papa. Tu tiens la pelle, Nino ? Oui, papa. Mila arrive près du bac. Elle marche sans bruit. Tu creuses avec moi ? Mila ne dit rien. Elle regarde ses mains. Le sable y luit un peu. On fait un puits. Nino ouvre la bouche trop vite. Les mots montent. Tu vois Mila, Nino ? Oui, papa.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Le sable est chaud. Un oiseau chante. [pause]</t>
+          <t>Le plastique du seau tape le rebord du bac. Ça fait toc, court et chaud. J'ai entendu le toc. Près du bac, Nino ? Oui, papa. Le sable sent le soleil. Papa pose le sac de goûter. Le sac fait un bruit de papier. Je déplie la couverture à carreaux. Les carreaux sont bleus et blancs. Elle est tiède, maman. Tu la sens, sous les genoux ? Oui, maman. Un oiseau gris picore près du banc. Au bord du bois, un &lt;emphasis&gt;éclat de banc&lt;/emphasis&gt; brille. Il brille, papa. Tu le vois, le petit point ? Oui, un petit point. Une cigale chante près des arbres. Elle chante fort. Le sable est chaud, Nino ? Oui, il brûle un peu. Je veux un puits, maintenant ! Un puits pour le seau rouge. Un puits dans le bac ? Oui. Bien creux. En ce moment, Nino s'assoit près du bac. Le seau rouge est tiède. Une pelle jaune est à côté. Le manche est un peu rêche. Il gratte, papa. Tu tiens la pelle, Nino ? Oui, papa. Mila arrive près du bac. Elle marche sans bruit. Tu creuses avec moi ? Mila ne dit rien. Elle regarde ses mains. Le sable y luit un peu. On fait un puits. Nino ouvre la bouche trop vite. Les mots montent. Tu vois Mila, Nino ? Oui, papa. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1254,10 +1254,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1278,28 +1278,32 @@
       <c r="AG2" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH2" s="2" t="inlineStr"/>
+      <c r="AH2" s="2" t="inlineStr">
+        <is>
+          <t>éclat de banc</t>
+        </is>
+      </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1308,10 +1312,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1322,21 +1326,37 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis élan; intensite=2; destinataire=enfant; sous_texte=il_veut_un_puits_maintenant; tempo=naturel puis resserré; sourire=léger puis large; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une cigale chante tout près du bac.
-narrateur|Le sable sent encore le soleil.
-narrateur|Un oiseau gris picore près du banc.
+          <t>narrateur|Le plastique du seau tape le rebord du bac.
+narrateur|Ça fait toc, court et chaud.
+enfant-m|J'ai entendu le toc.
+papa|Près du bac, Nino ?
+enfant-m|Oui, papa.
+narrateur|Le sable sent le soleil.
 narrateur|Papa pose le sac de goûter.
 narrateur|Le sac fait un bruit de papier.
-narrateur|Maman déplie une couverture à carreaux.
+maman|Je déplie la couverture à carreaux.
 narrateur|Les carreaux sont bleus et blancs.
-papa|Tu as entendu la cigale, Nino ?
+enfant-m|Elle est tiède, maman.
+maman|Tu la sens, sous les genoux ?
+enfant-m|Oui, maman.
+narrateur|Un oiseau gris picore près du banc.
+narrateur|Au bord du bois, un éclat de banc brille.
+enfant-m|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-m|Oui, un petit point.
+narrateur|Une cigale chante près des arbres.
 enfant-m|Elle chante fort.
-maman|Le sable est encore chaud.
-enfant-m|Je veux un puits.
-enfant-m|Pour le seau rouge.
+maman|Le sable est chaud, Nino ?
+enfant-m|Oui, il brûle un peu.
+enfant-m|Je veux un puits, maintenant !
+enfant-m|Un puits pour le seau rouge.
 papa|Un puits dans le bac ?
 enfant-m|Oui.
 enfant-m|Bien creux.
@@ -1344,10 +1364,20 @@
 narrateur|Le seau rouge est tiède.
 narrateur|Une pelle jaune est à côté.
 narrateur|Le manche est un peu rêche.
-narrateur|Mila est déjà là.
-narrateur|Elle parle peu.
+enfant-m|Il gratte, papa.
+papa|Tu tiens la pelle, Nino ?
+enfant-m|Oui, papa.
+narrateur|Mila arrive près du bac.
+narrateur|Elle marche sans bruit.
+enfant-m|Tu creuses avec moi ?
+narrateur|Mila ne dit rien.
 narrateur|Elle regarde ses mains.
-narrateur|Le sable y brille un peu.</t>
+narrateur|Le sable y luit un peu.
+enfant-m|On fait un puits.
+narrateur|Nino ouvre la bouche trop vite.
+narrateur|Les mots montent.
+papa|Tu vois Mila, Nino ?
+enfant-m|Oui, papa.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1379,17 +1409,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Nino a envie de tout expliquer. Le puits. L'eau. Le seau. Les mots restent un moment. On peut attendre. Tu peux tendre un jouet. Nino tient le seau rouge. Le plastique est tiède. Mila ne dit rien. Un grain de sable roule sur le bord. La cigale chante encore. Nino reste assis.</t>
+          <t>Nino a envie de tout expliquer. Le puits ! L'eau ! Le seau ! Les mots se bousculent dans sa bouche. Il pousse le seau vers Mila. Prends-le, maintenant ! Le seau penche trop. Le sable tombe sur le bord. Mila retire les doigts. Elle ne dit rien. Oh. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Elle a retiré les mains, Nino ? Oui, papa. Tes mains tiennent le seau, Nino ? Un peu, maman. L'éclat de banc tremble, puis tient. Mila tape le sable du doigt. Elle reste là, papa. Tu la vois, près du bac ? Oui. Papa s'accroupit à la même hauteur. Nino regarde papa.</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino a envie de tout expliquer. Le puits. L'eau. Le seau. Les mots restent un moment. On peut attendre. Tu peux tendre un jouet. Nino tient le seau rouge. Le plastique est tiède. Mila ne dit rien. Un grain de sable roule sur le bord. La cigale chante encore. Nino reste assis.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Nino a envie de tout expliquer. Le puits ! L'eau ! Le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt; ! Les mots se bousculent dans sa bouche. Il pousse le seau vers Mila. Prends-le, maintenant ! Le seau penche trop. Le sable tombe sur le bord. Mila retire les doigts. Elle ne dit rien. Oh. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Elle a retiré les mains, Nino ? Oui, papa. Tes mains tiennent le seau, Nino ? Un peu, maman. L'éclat de banc tremble, puis tient. Mila tape le sable du doigt. Elle reste là, papa. Tu la vois, près du bac ? Oui. Papa s'accroupit à la même hauteur. Nino regarde papa.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Léa est au parc avec maman. Adam est près du bac. Il parle peu. Léa veut jouer. Maman dit : on attend. On n'imite pas. On peut tendre un jouet. On ne force pas la parole. Léa tend le seau. Elle attend. Adam touche le seau. Il ne dit rien. Léa sourit. Elle ne force pas la parole. Plus tard, Adam dit : sable. Léa a su &lt;emphasis&gt;attendre&lt;/emphasis&gt;. Elle a tendu un jouet. [pause]</t>
+          <t>&lt;low-pitch&gt;Nino a envie de tout expliquer. Le puits ! L'eau ! Le &lt;emphasis&gt;seau&lt;/emphasis&gt; ! Les mots se bousculent dans sa bouche. Il pousse le seau vers Mila. Prends-le, maintenant ! Le seau penche trop. Le sable tombe sur le bord. Mila retire les doigts. Elle ne dit rien. Oh. Le sourire de Nino disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. Elle a retiré les mains, Nino ? Oui, papa. Tes mains tiennent le seau, Nino ? Un peu, maman. L'éclat de banc tremble, puis tient. Mila tape le sable du doigt. Elle reste là, papa. Tu la vois, près du bac ? Oui. Papa s'accroupit à la même hauteur. Nino regarde papa.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
@@ -1436,7 +1466,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1444,22 +1474,26 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE3" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE3" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF3" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1470,30 +1504,30 @@
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
-          <t>attendre</t>
+          <t>seau</t>
         </is>
       </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>300</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1502,36 +1536,53 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.92</v>
+        <v>0.93</v>
       </c>
       <c r="AS3" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT3" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU3" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV3" s="2" t="inlineStr"/>
+      <c r="AV3" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=élan puis découragement; intensite=2; destinataire=enfant; sous_texte=mila_retire_les_doigts_ne_dit_rien; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW3" t="inlineStr">
         <is>
           <t>narrateur|Nino a envie de tout expliquer.
-narrateur|Le puits.
-narrateur|L'eau.
-narrateur|Le seau.
-narrateur|Les mots restent un moment.
-maman|On peut attendre.
-papa|Tu peux tendre un jouet.
-narrateur|Nino tient le seau rouge.
-narrateur|Le plastique est tiède.
-narrateur|Mila ne dit rien.
-narrateur|Un grain de sable roule sur le bord.
-narrateur|La cigale chante encore.
-narrateur|Nino reste assis.</t>
+enfant-m|Le puits !
+enfant-m|L'eau !
+enfant-m|Le seau !
+narrateur|Les mots se bousculent dans sa bouche.
+narrateur|Il pousse le seau vers Mila.
+enfant-m|Prends-le, maintenant !
+narrateur|Le seau penche trop.
+narrateur|Le sable tombe sur le bord.
+narrateur|Mila retire les doigts.
+narrateur|Elle ne dit rien.
+enfant-m|Oh.
+narrateur|Le sourire de Nino disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+papa|Elle a retiré les mains, Nino ?
+enfant-m|Oui, papa.
+maman|Tes mains tiennent le seau, Nino ?
+enfant-m|Un peu, maman.
+narrateur|L'éclat de banc tremble, puis tient.
+narrateur|Mila tape le sable du doigt.
+enfant-m|Elle reste là, papa.
+papa|Tu la vois, près du bac ?
+enfant-m|Oui.
+narrateur|Papa s'accroupit à la même hauteur.
+narrateur|Nino regarde papa.</t>
         </is>
       </c>
       <c r="AX3" t="inlineStr">
@@ -1568,12 +1619,12 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Mila parle peu. Que fait Nino ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Mila parle peu. Que fait &lt;emphasis level="moderate"&gt;Nino&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Adam parle peu. Que fait Léa ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Mila parle peu. Que fait &lt;emphasis&gt;Nino&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1636,7 +1687,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1647,7 +1698,7 @@
         <v>0.86</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.27</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1662,34 +1713,38 @@
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH4" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>Nino</t>
+        </is>
+      </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1704,17 +1759,17 @@
         <v>0.86</v>
       </c>
       <c r="AS4" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT4" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=mila_parle_peu_que_fait_nino; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
@@ -1747,17 +1802,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Nino tend le seau. Pour le puits. Il attend. Mila touche le seau. Elle ne dit rien. On ne force pas la parole. Le seau peut suffire. Mila prend le seau. Elle le remplit. Le sable fait un bruit doux. Nino creuse avec la pelle jaune. Un trou rond s'ouvre. Mila verse le seau. Le puits grandit. Encore un peu. Mila verse encore. Puis elle dit tout bas. Puits. Puits. Tu as su attendre. Bravo, Nino. Maman ouvre la gourde. Un filet d'eau tombe dans le trou. Le fond devient sombre. Eau. Eau.</t>
+          <t>Nino veut tout dire, tout de suite. Je t'explique, maintenant ! Il avance trop vite vers Mila. Les mots se bousculent. Mila recule un peu. Oh. Le sourire ne revient pas. Nino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le seau, un instant. Il écoute la cigale. Tu veux le puits avec Mila ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le seau, puis la pelle. D'accord. Nino tend le seau, sans se presser. Il reste un moment, les mains ouvertes. Mila souffle. Elle tend les mains, sans parler. Oui. Mila prend le seau. Merci, Nino. Papa a vu les deux, près du bac. Le plastique est tiède, sous les doigts. Il est chaud. Mila le remplit. Nino creuse avec la pelle jaune. Un trou rond s'ouvre. Mila verse le seau. Le puits grandit. Le puits. Puits. Puits. Tes mains sont au chaud, Nino ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Nino tend le seau. Pour le puits. Il attend. Mila touche le seau. Elle ne dit rien. On ne force pas la parole. Le seau peut suffire. Mila prend le seau. Elle le remplit. Le sable fait un bruit doux. Nino creuse avec la pelle jaune. Un trou rond s'ouvre. Mila verse le seau. Le puits grandit. Encore un peu. Mila verse encore. Puis elle dit tout bas. Puits. Puits. Tu as su attendre. Bravo, Nino. Maman ouvre la gourde. Un filet d'eau tombe dans le trou. Le fond devient sombre. Eau. Eau.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Nino veut tout dire, tout de suite. Je t'explique, maintenant ! Il avance trop vite vers Mila. Les mots se bousculent. Mila recule un peu. Oh. Le sourire ne revient pas. Nino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le &lt;emphasis level="moderate"&gt;seau&lt;/emphasis&gt;, un instant. Il écoute la cigale. Tu veux le puits avec Mila ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le seau, puis la pelle. D'accord. Nino tend le seau, sans se presser. Il reste un moment, les mains ouvertes. Mila souffle. Elle tend les mains, sans parler. Oui. Mila prend le seau. Merci, Nino. Papa a vu les deux, près du bac. Le plastique est tiède, sous les doigts. Il est chaud. Mila le remplit. Nino creuse avec la pelle jaune. Un trou rond s'ouvre. Mila verse le seau. Le puits grandit. Le puits. Puits. Puits. Tes mains sont au chaud, Nino ? Un peu, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Léa a attendu. Elle a tendu un jouet. Elle n'a &lt;emphasis&gt;pas&lt;/emphasis&gt; forcé la parole. [pause]</t>
+          <t>Nino veut tout dire, tout de suite. Je t'explique, maintenant ! Il avance trop vite vers Mila. Les mots se bousculent. Mila recule un peu. Oh. Le sourire ne revient pas. Nino refuse de foncer. Il referme la bouche. Personne ne parle. Il observe le &lt;emphasis&gt;seau&lt;/emphasis&gt;, un instant. Il écoute la cigale. Tu veux le puits avec Mila ? Papa reste à la même hauteur. Papa, on fait quoi ? On pose le seau, puis la pelle. D'accord. Nino tend le seau, sans se presser. Il reste un moment, les mains ouvertes. Mila souffle. Elle tend les mains, sans parler. Oui. Mila prend le seau. Merci, Nino. Papa a vu les deux, près du bac. Le plastique est tiède, sous les doigts. Il est chaud. Mila le remplit. Nino creuse avec la pelle jaune. Un trou rond s'ouvre. Mila verse le seau. Le puits grandit. Le puits. Puits. Puits. Tes mains sont au chaud, Nino ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1804,7 +1859,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1812,10 +1867,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1838,30 +1893,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>pas</t>
+          <t>seau</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1870,10 +1925,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1886,37 +1941,48 @@
       </c>
       <c r="AV5" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=il_refuse_de_foncer_tend_attend; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Nino tend le seau.
-enfant-m|Pour le puits.
-narrateur|Il attend.
-narrateur|Mila touche le seau.
-narrateur|Elle ne dit rien.
-maman|On ne force pas la parole.
-papa|Le seau peut suffire.
+          <t>narrateur|Nino veut tout dire, tout de suite.
+enfant-m|Je t'explique, maintenant !
+narrateur|Il avance trop vite vers Mila.
+narrateur|Les mots se bousculent.
+narrateur|Mila recule un peu.
+enfant-m|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Nino refuse de foncer.
+narrateur|Il referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Il observe le seau, un instant.
+narrateur|Il écoute la cigale.
+papa|Tu veux le puits avec Mila ?
+narrateur|Papa reste à la même hauteur.
+enfant-m|Papa, on fait quoi ?
+papa|On pose le seau, puis la pelle.
+enfant-m|D'accord.
+narrateur|Nino tend le seau, sans se presser.
+narrateur|Il reste un moment, les mains ouvertes.
+narrateur|Mila souffle.
+narrateur|Elle tend les mains, sans parler.
+copine|Oui.
 narrateur|Mila prend le seau.
-narrateur|Elle le remplit.
-narrateur|Le sable fait un bruit doux.
+papa|Merci, Nino.
+narrateur|Papa a vu les deux, près du bac.
+maman|Le plastique est tiède, sous les doigts.
+enfant-m|Il est chaud.
+narrateur|Mila le remplit.
 narrateur|Nino creuse avec la pelle jaune.
 narrateur|Un trou rond s'ouvre.
 narrateur|Mila verse le seau.
 narrateur|Le puits grandit.
-enfant-m|Encore un peu.
-narrateur|Mila verse encore.
-narrateur|Puis elle dit tout bas.
-enfant-f|Puits.
+enfant-m|Le puits.
+copine|Puits.
 enfant-m|Puits.
-papa|Tu as su attendre.
-papa|Bravo, Nino.
-narrateur|Maman ouvre la gourde.
-narrateur|Un filet d'eau tombe dans le trou.
-narrateur|Le fond devient sombre.
-enfant-f|Eau.
-enfant-m|Eau.</t>
+maman|Tes mains sont au chaud, Nino ?
+enfant-m|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX5" t="inlineStr">
@@ -1948,17 +2014,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Le puits brille un peu. Le bord est encore chaud. La cigale chante encore. Une compote ? Mila secoue la tête. D'accord. D'accord. Tu as fini le puits, Nino ? Oui, maman. Il a de l'eau. Papa plie un coin de couverture. Nino pose le seau à l'ombre. Mila reste près du trou. Elle regarde l'eau. Un grain colle encore à son genou. L'oiseau s'est envolé. Le bac reste chaud. La couverture à carreaux est un peu sablée. Le sable colle.</t>
+          <t>Maman ouvre la gourde. L'eau, maintenant ! Nino envoie la gourde trop vite. Un filet penche hors du trou. Ça tombe ! Dis-le, Mila ! Mila serre les lèvres. Nino avance les mains, trop vite. Puis il s'arrête net. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le banc, un instant. Il écoute l'oiseau près du bois. Au bord du banc, un éclat de banc luit. Là, sur le banc. Tu prends la gourde, Mila ? Mila ne dit rien. Elle tend les mains, sans parler. Oui. Nino passe la gourde, sans se presser. Mila verse, plus lentement. Le fond devient sombre. Eau. Eau. Tu la vois, l'eau ? Oui, papa. Le puits est creux, Nino ? Oui, maman. Ils restent près du trou. La couverture à carreaux est un peu sablée. Le puits tient, Nino ? Oui, papa. Un rayon passe sur le seau rouge. Il allume le puits.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Le puits brille un peu. Le bord est encore chaud. La cigale chante encore. Une compote ? Mila secoue la tête. D'accord. D'accord. Tu as fini le puits, Nino ? Oui, maman. Il a de l'eau. Papa plie un coin de couverture. Nino pose le seau à l'ombre. Mila reste près du trou. Elle regarde l'eau. Un grain colle encore à son genou. L'oiseau s'est envolé. Le bac reste chaud. La couverture à carreaux est un peu sablée. Le sable colle.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman ouvre la gourde. L'eau, maintenant ! Nino envoie la gourde trop vite. Un filet penche hors du trou. Ça tombe ! Dis-le, Mila ! Mila serre les lèvres. Nino avance les mains, trop vite. Puis il s'arrête net. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le banc, un instant. Il écoute l'oiseau près du bois. Au bord du banc, un &lt;emphasis level="moderate"&gt;éclat de banc&lt;/emphasis&gt; luit. Là, sur le banc. Tu prends la gourde, Mila ? Mila ne dit rien. Elle tend les mains, sans parler. Oui. Nino passe la gourde, sans se presser. Mila verse, plus lentement. Le fond devient sombre. Eau. Eau. Tu la vois, l'eau ? Oui, papa. Le puits est creux, Nino ? Oui, maman. Ils restent près du trou. La couverture à carreaux est un peu sablée. Le puits tient, Nino ? Oui, papa. Un rayon passe sur le seau rouge. Il allume le puits.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Maman range le seau. Léa donne la &lt;emphasis&gt;main&lt;/emphasis&gt;. [pause]</t>
+          <t>Maman ouvre la gourde. L'eau, maintenant ! Nino envoie la gourde trop vite. Un filet penche hors du trou. Ça tombe ! Dis-le, Mila ! Mila serre les lèvres. Nino avance les mains, trop vite. Puis il s'arrête net. Nino refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Il observe le banc, un instant. Il écoute l'oiseau près du bois. Au bord du banc, un &lt;emphasis&gt;éclat de banc&lt;/emphasis&gt; luit. Là, sur le banc. Tu prends la gourde, Mila ? Mila ne dit rien. Elle tend les mains, sans parler. Oui. Nino passe la gourde, sans se presser. Mila verse, plus lentement. Le fond devient sombre. Eau. Eau. Tu la vois, l'eau ? Oui, papa. Le puits est creux, Nino ? Oui, maman. Ils restent près du trou. La couverture à carreaux est un peu sablée. Le puits tient, Nino ? Oui, papa. Un rayon passe sur le seau rouge. Il allume le puits. [pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2005,7 +2071,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2013,10 +2079,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.1</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2039,30 +2105,30 @@
       </c>
       <c r="AH6" s="2" t="inlineStr">
         <is>
-          <t>main</t>
+          <t>éclat de banc</t>
         </is>
       </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2071,10 +2137,10 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS6" s="2" t="n">
         <v>100</v>
@@ -2085,28 +2151,53 @@
       <c r="AU6" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=gourde_trop_vite_il_s_arrete; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Le puits brille un peu.
-narrateur|Le bord est encore chaud.
-narrateur|La cigale chante encore.
-maman|Une compote ?
-narrateur|Mila secoue la tête.
-enfant-m|D'accord.
-papa|D'accord.
-maman|Tu as fini le puits, Nino ?
+          <t>narrateur|Maman ouvre la gourde.
+enfant-m|L'eau, maintenant !
+narrateur|Nino envoie la gourde trop vite.
+narrateur|Un filet penche hors du trou.
+enfant-m|Ça tombe !
+enfant-m|Dis-le, Mila !
+narrateur|Mila serre les lèvres.
+narrateur|Nino avance les mains, trop vite.
+narrateur|Puis il s'arrête net.
+narrateur|Nino refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Il observe le banc, un instant.
+narrateur|Il écoute l'oiseau près du bois.
+narrateur|Au bord du banc, un éclat de banc luit.
+enfant-m|Là, sur le banc.
+enfant-m|Tu prends la gourde, Mila ?
+narrateur|Mila ne dit rien.
+narrateur|Elle tend les mains, sans parler.
+copine|Oui.
+narrateur|Nino passe la gourde, sans se presser.
+narrateur|Mila verse, plus lentement.
+narrateur|Le fond devient sombre.
+copine|Eau.
+enfant-m|Eau.
+papa|Tu la vois, l'eau ?
+enfant-m|Oui, papa.
+maman|Le puits est creux, Nino ?
 enfant-m|Oui, maman.
-enfant-m|Il a de l'eau.
-narrateur|Papa plie un coin de couverture.
-narrateur|Nino pose le seau à l'ombre.
-narrateur|Mila reste près du trou.
-narrateur|Elle regarde l'eau.
-narrateur|Un grain colle encore à son genou.
-papa|L'oiseau s'est envolé.
-narrateur|Le bac reste chaud.
+narrateur|Ils restent près du trou.
 narrateur|La couverture à carreaux est un peu sablée.
-enfant-m|Le sable colle.</t>
+papa|Le puits tient, Nino ?
+enfant-m|Oui, papa.
+maman|Un rayon passe sur le seau rouge.
+enfant-m|Il allume le puits.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>enfants_parc</t>
         </is>
       </c>
     </row>
@@ -2133,17 +2224,17 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>On a fait un puits. Avec le seau rouge. L'eau est au fond.</t>
+          <t>Ils restent près du bac. Une compote, Nino ? Mila secoue la tête. D'accord. D'accord. Tu as fini le puits, Nino ? Oui, maman. Il a de l'eau. Tu souffles sur le bord ? Oui, papa. Nino souffle, un peu de sable vole. Le sable est chaud. Tu le sens, le sable ? Oui, maman. Le puits reste un peu, rond. Il a tenu, dans le bac. Puits. Le seau est à l'ombre, sous le banc. Le puits fait une petite ombre. On y remet de l'eau, après. Un éclat de banc tient près de l'oiseau.</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>On a fait un puits. Avec le seau rouge. L'eau est au fond.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du bac. Une compote, Nino ? Mila secoue la tête. D'accord. D'accord. Tu as fini le puits, Nino ? Oui, maman. Il a de l'eau. Tu souffles sur le bord ? Oui, papa. Nino souffle, un peu de sable vole. Le sable est chaud. Tu le sens, le sable ? Oui, maman. Le puits reste un peu, rond. Il a tenu, dans le bac. Puits. Le seau est à l'ombre, sous le banc. Le puits fait une petite ombre. On y remet de l'eau, après. Un &lt;emphasis level="moderate"&gt;éclat de banc&lt;/emphasis&gt; tient près de l'oiseau.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du bac. Une compote, Nino ? Mila secoue la tête. D'accord. D'accord. Tu as fini le puits, Nino ? Oui, maman. Il a de l'eau. Tu souffles sur le bord ? Oui, papa. Nino souffle, un peu de sable vole. Le sable est chaud. Tu le sens, le sable ? Oui, maman. Le puits reste un peu, rond. Il a tenu, dans le bac. Puits. Le seau est à l'ombre, sous le banc. Le puits fait une petite ombre. On y remet de l'eau, après. Un &lt;emphasis&gt;éclat de banc&lt;/emphasis&gt; tient près de l'oiseau.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -2190,15 +2281,15 @@
         </is>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z7" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA7" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB7" s="2" t="n">
         <v>1.28</v>
@@ -2210,12 +2301,12 @@
       </c>
       <c r="AD7" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE7" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF7" s="2" t="inlineStr">
@@ -2224,17 +2315,21 @@
         </is>
       </c>
       <c r="AG7" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH7" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH7" s="2" t="inlineStr">
+        <is>
+          <t>éclat de banc</t>
+        </is>
+      </c>
       <c r="AI7" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ7" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL7" s="2" t="inlineStr">
         <is>
@@ -2243,11 +2338,11 @@
       </c>
       <c r="AM7" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO7" s="2" t="inlineStr"/>
       <c r="AP7" s="2" t="inlineStr">
@@ -2256,26 +2351,48 @@
         </is>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS7" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT7" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU7" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV7" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV7" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_pres_de_l_oiseau; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW7" t="inlineStr">
         <is>
-          <t>enfant-m|On a fait un puits.
-maman|Avec le seau rouge.
-papa|L'eau est au fond.</t>
+          <t>narrateur|Ils restent près du bac.
+maman|Une compote, Nino ?
+narrateur|Mila secoue la tête.
+enfant-m|D'accord.
+papa|D'accord.
+maman|Tu as fini le puits, Nino ?
+enfant-m|Oui, maman.
+enfant-m|Il a de l'eau.
+papa|Tu souffles sur le bord ?
+enfant-m|Oui, papa.
+narrateur|Nino souffle, un peu de sable vole.
+enfant-m|Le sable est chaud.
+maman|Tu le sens, le sable ?
+enfant-m|Oui, maman.
+papa|Le puits reste un peu, rond.
+enfant-m|Il a tenu, dans le bac.
+copine|Puits.
+narrateur|Le seau est à l'ombre, sous le banc.
+narrateur|Le puits fait une petite ombre.
+enfant-m|On y remet de l'eau, après.
+narrateur|Un éclat de banc tient près de l'oiseau.</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2360,6 +2477,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>